<commit_message>
feat(comp-tracker): rebuild workflow with cliclick stack + run April 2026
- Rewrote steps 01-04: replaced browser_batch with cliclick + execute_javascript + get_page_content
- Added Show visuals as tables protocol (mandatory Step 0b) - persists across page navigations
- Added Date slicer protocol - set once on Customer Distribution, carries to all pages
- Documented coordinate system: screen_y = 154 + page_y (window_y:33 + chrome_ui:121)
- Fixed Row 14 pro-rated growth formula for Comp 2 Region sheet
- Added TOTAL LEADS row protection in step-05 (insert before, not after)
- Added row formatting copy protocol via AppleScript paste special in step-05
- Created step-07-prompt-comp3.md (new - Comp 3 strategic activities prompt)
- Updated workflow.md: new state keys, click stack docs, updated known behavior table
- Updated Comp Tracker: April 2026 YTD revenue + GM% for 9 named accounts, Comp 2 Jan-Mar data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/systems/compensation/2026 Comp Tracker.xlsx
+++ b/systems/compensation/2026 Comp Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://improving-my.sharepoint.com/personal/david_ohara_improving_com/Documents/IES/systems/compensation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_DEF1EA21AFB58EC042CA4DA58E535AFA914832E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13EFB9B3-34C1-9E48-920D-D8150CAA4F6B}"/>
+  <xr:revisionPtr revIDLastSave="112" documentId="11_DEF1EA21AFB58EC042CA4DA58E535AFA914832E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F63E8F9-2DDE-A549-8F11-6CB57694DB5D}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="21380" windowHeight="11120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="21380" windowHeight="11120" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="167">
   <si>
     <t>2026 REGIONAL DIRECTOR COMPENSATION TRACKER</t>
   </si>
@@ -514,7 +514,34 @@
     <t>Integrated Financial Settlements</t>
   </si>
   <si>
-    <t>TOTAL LEADS</t>
+    <t>Cardinal IT Solutions (Kashif)</t>
+  </si>
+  <si>
+    <t>Steve Hall</t>
+  </si>
+  <si>
+    <t>Derek Nwamadi</t>
+  </si>
+  <si>
+    <t>Paragon Brokerage</t>
+  </si>
+  <si>
+    <t>Me</t>
+  </si>
+  <si>
+    <t>Kubota</t>
+  </si>
+  <si>
+    <t>Nexben</t>
+  </si>
+  <si>
+    <t>Specialty Capital</t>
+  </si>
+  <si>
+    <t>Shalini Arora</t>
+  </si>
+  <si>
+    <t>Birgo</t>
   </si>
 </sst>
 </file>
@@ -811,7 +838,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -938,11 +965,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -954,12 +982,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1257,39 +1279,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="77" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
+      <c r="A1" s="76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="78" t="s">
+      <c r="A2" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="79" t="s">
+      <c r="B4" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
@@ -1309,7 +1331,7 @@
       </c>
       <c r="C6" s="5">
         <f>'Comp 1 - BoB'!H38</f>
-        <v>-1</v>
+        <v>-0.76101567311789919</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -1361,7 +1383,7 @@
       </c>
       <c r="C10" s="7">
         <f>SUM(C5:C9)</f>
-        <v>179999.36129753533</v>
+        <v>179999.60028186222</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
@@ -1382,14 +1404,14 @@
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="79" t="s">
+      <c r="B13" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79"/>
-      <c r="E13" s="79"/>
-      <c r="F13" s="79"/>
-      <c r="G13" s="79"/>
+      <c r="C13" s="78"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="78"/>
+      <c r="F13" s="78"/>
+      <c r="G13" s="78"/>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
@@ -1573,28 +1595,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="80"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="81" t="s">
+      <c r="A2" s="80" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
     </row>
     <row r="4" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="18" t="s">
@@ -1630,11 +1652,15 @@
         <v>476120</v>
       </c>
       <c r="E5" s="22"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="24" t="str">
+      <c r="F5" s="21">
+        <v>122160</v>
+      </c>
+      <c r="G5" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="H5" s="24">
         <f t="shared" ref="H5:H24" si="0">IF(D5=0,"-",IF(F5=0,"-",(F5-D5)/D5))</f>
-        <v>-</v>
+        <v>-0.74342602705200367</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1648,11 +1674,15 @@
         <v>925267</v>
       </c>
       <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="29" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F6" s="27">
+        <v>209300</v>
+      </c>
+      <c r="G6" s="28">
+        <v>0.21</v>
+      </c>
+      <c r="H6" s="29">
+        <f t="shared" si="0"/>
+        <v>-0.77379502349051676</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1666,11 +1696,15 @@
         <v>1093108.77</v>
       </c>
       <c r="E7" s="22"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F7" s="21">
+        <v>277859</v>
+      </c>
+      <c r="G7" s="23">
+        <v>0.4</v>
+      </c>
+      <c r="H7" s="24">
+        <f t="shared" si="0"/>
+        <v>-0.74580846149464153</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1684,11 +1718,15 @@
         <v>5024642</v>
       </c>
       <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F8" s="27">
+        <v>1131915</v>
+      </c>
+      <c r="G8" s="28">
+        <v>0.4</v>
+      </c>
+      <c r="H8" s="29">
+        <f t="shared" si="0"/>
+        <v>-0.77472723429848334</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1720,11 +1758,15 @@
         <v>628655.41</v>
       </c>
       <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="29" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F10" s="27">
+        <v>105947</v>
+      </c>
+      <c r="G10" s="28">
+        <v>0.38</v>
+      </c>
+      <c r="H10" s="29">
+        <f t="shared" si="0"/>
+        <v>-0.83147047123956197</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1738,11 +1780,15 @@
         <v>2760096.23</v>
       </c>
       <c r="E11" s="22"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F11" s="21">
+        <v>771212</v>
+      </c>
+      <c r="G11" s="23">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="H11" s="24">
+        <f t="shared" si="0"/>
+        <v>-0.7205851043823932</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1756,11 +1802,15 @@
         <v>1004738</v>
       </c>
       <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F12" s="27">
+        <v>264730</v>
+      </c>
+      <c r="G12" s="28">
+        <v>0.26</v>
+      </c>
+      <c r="H12" s="29">
+        <f t="shared" si="0"/>
+        <v>-0.73651837593482083</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1774,11 +1824,15 @@
         <v>659367.62</v>
       </c>
       <c r="E13" s="22"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F13" s="21">
+        <v>145356</v>
+      </c>
+      <c r="G13" s="23">
+        <v>0.27</v>
+      </c>
+      <c r="H13" s="24">
+        <f t="shared" si="0"/>
+        <v>-0.77955241417526688</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1792,11 +1846,15 @@
         <v>770198.75</v>
       </c>
       <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="29" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F14" s="27">
+        <v>171908</v>
+      </c>
+      <c r="G14" s="28">
+        <v>0.22</v>
+      </c>
+      <c r="H14" s="29">
+        <f t="shared" si="0"/>
+        <v>-0.77680046871018682</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1961,27 +2019,27 @@
       </c>
       <c r="F25" s="34">
         <f>SUM(F5:F24)</f>
-        <v>0</v>
-      </c>
-      <c r="G25" s="35" t="str">
+        <v>3200387</v>
+      </c>
+      <c r="G25" s="35">
         <f>IF(F25=0,"-",SUMPRODUCT(F5:F24,G5:G24)/F25)</f>
-        <v>-</v>
+        <v>0.32511615001560751</v>
       </c>
       <c r="H25" s="35">
         <f>IF(D25=0,"-",(F25-D25)/D25)</f>
-        <v>-1</v>
+        <v>-0.76101567311789919</v>
       </c>
     </row>
     <row r="28" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="79" t="s">
+      <c r="B28" s="78" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
-      <c r="E28" s="79"/>
-      <c r="F28" s="79"/>
-      <c r="G28" s="79"/>
-      <c r="H28" s="79"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="78"/>
       <c r="I28" s="36"/>
     </row>
     <row r="29" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2270,16 +2328,16 @@
       </c>
       <c r="H38" s="24">
         <f>H25</f>
-        <v>-1</v>
+        <v>-0.76101567311789919</v>
       </c>
     </row>
     <row r="39" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="H39" s="24" t="str">
+      <c r="H39" s="24">
         <f>G25</f>
-        <v>-</v>
+        <v>0.32511615001560751</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2318,42 +2376,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="74" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82"/>
-      <c r="O1" s="82"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="N1" s="74"/>
+      <c r="O1" s="74"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="75" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="83"/>
-      <c r="J2" s="83"/>
-      <c r="K2" s="83"/>
-      <c r="L2" s="83"/>
-      <c r="M2" s="83"/>
-      <c r="N2" s="83"/>
-      <c r="O2" s="83"/>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
     </row>
     <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
@@ -2654,55 +2712,55 @@
         <v>97</v>
       </c>
       <c r="C14" s="51">
-        <f t="shared" ref="C14:O14" si="3">IF($C$4=0,"-",(C13-$C$4)/$C$4)</f>
-        <v>-0.92464520775623271</v>
+        <f t="shared" ref="C14:N14" si="3">(C13-($C$4*(COLUMN()-2)/12))/($C$4*(COLUMN()-2)/12)</f>
+        <v>-9.5742493074792295E-2</v>
       </c>
       <c r="D14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.84923180055401659</v>
+        <v>-9.5390803324099771E-2</v>
       </c>
       <c r="E14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-7.1979335180055407E-2</v>
       </c>
       <c r="F14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.30398450138504157</v>
       </c>
       <c r="G14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.44318760110803324</v>
       </c>
       <c r="H14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.53598966759002775</v>
       </c>
       <c r="I14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.60227685793430941</v>
       </c>
       <c r="J14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.65199225069252076</v>
       </c>
       <c r="K14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.6906597783933518</v>
       </c>
       <c r="L14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.72159380055401656</v>
       </c>
       <c r="M14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.74690345504910605</v>
       </c>
       <c r="N14" s="51">
         <f t="shared" si="3"/>
         <v>-0.76799483379501388</v>
       </c>
       <c r="O14" s="42">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="O14" si="4">IF($C$4=0,"-",(O13-$C$4)/$C$4)</f>
         <v>-0.53598966759002775</v>
       </c>
     </row>
@@ -2765,22 +2823,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="81" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="85" t="s">
+      <c r="A2" s="82" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
@@ -2934,26 +2992,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="83" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="84" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="59" t="s">
@@ -3253,7 +3316,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3263,20 +3326,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="85" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="86" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="89"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
     </row>
     <row r="3" spans="1:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3612,14 +3675,116 @@
       <c r="D27" s="70"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="74" t="s">
+      <c r="A28" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B28" s="69">
+        <v>46066</v>
+      </c>
+      <c r="C28" s="70" t="s">
         <v>157</v>
       </c>
-      <c r="B28" s="75">
-        <v>23</v>
-      </c>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
+      <c r="D28" s="70" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B29" s="69">
+        <v>46069</v>
+      </c>
+      <c r="C29" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" s="70" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B30" s="69">
+        <v>46070</v>
+      </c>
+      <c r="C30" s="70" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" s="70" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B31" s="69">
+        <v>46084</v>
+      </c>
+      <c r="C31" s="70" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="70" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B32" s="69">
+        <v>46086</v>
+      </c>
+      <c r="C32" s="70" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" s="70" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B33" s="69">
+        <v>46093</v>
+      </c>
+      <c r="C33" s="70" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="70" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B34" s="69">
+        <v>46114</v>
+      </c>
+      <c r="C34" s="70" t="s">
+        <v>164</v>
+      </c>
+      <c r="D34" s="70" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="68">
+        <v>2026</v>
+      </c>
+      <c r="B35" s="69">
+        <v>46118</v>
+      </c>
+      <c r="C35" s="70" t="s">
+        <v>166</v>
+      </c>
+      <c r="D35" s="70" t="s">
+        <v>127</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
chore: cleanup temp artifacts and update tracked files
- Remove .DS_Store artifacts from workspace
- Remove FUSE hidden files from skills directory
- Update .gitignore rules for temp cleanup
- Refresh compensation tracker snapshot
- Update invintory MCP export script

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/systems/compensation/2026 Comp Tracker.xlsx
+++ b/systems/compensation/2026 Comp Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://improving-my.sharepoint.com/personal/david_ohara_improving_com/Documents/IES/systems/compensation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="112" documentId="11_DEF1EA21AFB58EC042CA4DA58E535AFA914832E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F63E8F9-2DDE-A549-8F11-6CB57694DB5D}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="11_DEF1EA21AFB58EC042CA4DA58E535AFA914832E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{977AC5BC-3375-E84C-95FC-809A92E38945}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="21380" windowHeight="11120" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="21380" windowHeight="11120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(chase,knox,rigby): July 14 session — scorecard, comp tracker, plaud ingest, workflow bugfix
- One Texas Scorecard updated through June 2026
- Comp tracker rerun with corrected PowerBI data (BoB $6.68M, -5.5% YoY)
- Plaud ingest: Kapil Dabi lunch + Steve Hall coffee ingested, 7 OmniFocus tasks
- Rigby fixed 2 plaud-ingest bugs: transcript placement, working memory path
- 3 error entries logged (Plaud skip, OOO fabrication, time calculation)
- Session cleanup: .DS_Store purged, working memory written
</commit_message>
<xml_diff>
--- a/systems/compensation/2026 Comp Tracker.xlsx
+++ b/systems/compensation/2026 Comp Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://improving-my.sharepoint.com/personal/david_ohara_improving_com/Documents/IES/systems/compensation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="11_DEF1EA21AFB58EC042CA4DA58E535AFA914832E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{977AC5BC-3375-E84C-95FC-809A92E38945}"/>
+  <xr:revisionPtr revIDLastSave="162" documentId="11_DEF1EA21AFB58EC042CA4DA58E535AFA914832E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8AF535E-18EF-5847-871A-A2DDE9FD0A24}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="21380" windowHeight="11120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28240" windowHeight="17240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="170">
   <si>
     <t>2026 REGIONAL DIRECTOR COMPENSATION TRACKER</t>
   </si>
@@ -542,6 +542,15 @@
   </si>
   <si>
     <t>Birgo</t>
+  </si>
+  <si>
+    <t>JSX</t>
+  </si>
+  <si>
+    <t>THL</t>
+  </si>
+  <si>
+    <t>Spring Line Advisory</t>
   </si>
 </sst>
 </file>
@@ -838,7 +847,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -965,23 +974,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1279,39 +1289,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="76" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
+      <c r="A1" s="78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="77" t="s">
+      <c r="A2" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="77"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="78" t="s">
+      <c r="B4" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="78"/>
-      <c r="D4" s="78"/>
-      <c r="E4" s="78"/>
-      <c r="F4" s="78"/>
-      <c r="G4" s="78"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
@@ -1331,7 +1341,7 @@
       </c>
       <c r="C6" s="5">
         <f>'Comp 1 - BoB'!H38</f>
-        <v>-0.76101567311789919</v>
+        <v>-0.50082741229286987</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -1344,7 +1354,7 @@
       </c>
       <c r="C7" s="5">
         <f>'Comp 2 - Region'!G18</f>
-        <v>0.36129753534359282</v>
+        <v>0.48779084467289063</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
@@ -1383,7 +1393,7 @@
       </c>
       <c r="C10" s="7">
         <f>SUM(C5:C9)</f>
-        <v>179999.60028186222</v>
+        <v>179999.98696343237</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
@@ -1404,14 +1414,14 @@
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="78" t="s">
+      <c r="B13" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="78"/>
-      <c r="D13" s="78"/>
-      <c r="E13" s="78"/>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
@@ -1462,7 +1472,7 @@
       </c>
       <c r="E16" s="15">
         <f>'Comp 2 - Region'!G17</f>
-        <v>-0.76799483379501388</v>
+        <v>-0.52741347645429359</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>19</v>
@@ -1595,28 +1605,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="75" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="80"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
     </row>
     <row r="4" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="18" t="s">
@@ -1653,14 +1663,14 @@
       </c>
       <c r="E5" s="22"/>
       <c r="F5" s="21">
-        <v>122160</v>
+        <v>249240</v>
       </c>
       <c r="G5" s="23">
         <v>0.25</v>
       </c>
       <c r="H5" s="24">
         <f t="shared" ref="H5:H24" si="0">IF(D5=0,"-",IF(F5=0,"-",(F5-D5)/D5))</f>
-        <v>-0.74342602705200367</v>
+        <v>-0.47651852474166179</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1675,14 +1685,14 @@
       </c>
       <c r="E6" s="27"/>
       <c r="F6" s="27">
-        <v>209300</v>
+        <v>338516</v>
       </c>
       <c r="G6" s="28">
         <v>0.21</v>
       </c>
       <c r="H6" s="29">
         <f t="shared" si="0"/>
-        <v>-0.77379502349051676</v>
+        <v>-0.63414236106983168</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1697,14 +1707,14 @@
       </c>
       <c r="E7" s="22"/>
       <c r="F7" s="21">
-        <v>277859</v>
+        <v>559386</v>
       </c>
       <c r="G7" s="23">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="H7" s="24">
         <f t="shared" si="0"/>
-        <v>-0.74580846149464153</v>
+        <v>-0.48826135572949436</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1719,14 +1729,14 @@
       </c>
       <c r="E8" s="27"/>
       <c r="F8" s="27">
-        <v>1131915</v>
+        <v>2308168</v>
       </c>
       <c r="G8" s="28">
         <v>0.4</v>
       </c>
       <c r="H8" s="29">
         <f t="shared" si="0"/>
-        <v>-0.77472723429848334</v>
+        <v>-0.54063035734685183</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1740,11 +1750,15 @@
         <v>32100</v>
       </c>
       <c r="E9" s="22"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="F9" s="21">
+        <v>161680</v>
+      </c>
+      <c r="G9" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="H9" s="24">
+        <f t="shared" si="0"/>
+        <v>4.0367601246105922</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1759,14 +1773,14 @@
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="27">
-        <v>105947</v>
+        <v>142502</v>
       </c>
       <c r="G10" s="28">
-        <v>0.38</v>
+        <v>0.5</v>
       </c>
       <c r="H10" s="29">
         <f t="shared" si="0"/>
-        <v>-0.83147047123956197</v>
+        <v>-0.77332255837900132</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1781,14 +1795,14 @@
       </c>
       <c r="E11" s="22"/>
       <c r="F11" s="21">
-        <v>771212</v>
+        <v>1677276</v>
       </c>
       <c r="G11" s="23">
         <v>0.28000000000000003</v>
       </c>
       <c r="H11" s="24">
         <f t="shared" si="0"/>
-        <v>-0.7205851043823932</v>
+        <v>-0.39231249194525364</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1803,14 +1817,14 @@
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="27">
-        <v>264730</v>
+        <v>532126</v>
       </c>
       <c r="G12" s="28">
         <v>0.26</v>
       </c>
       <c r="H12" s="29">
         <f t="shared" si="0"/>
-        <v>-0.73651837593482083</v>
+        <v>-0.47038332381177977</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1825,14 +1839,14 @@
       </c>
       <c r="E13" s="22"/>
       <c r="F13" s="21">
-        <v>145356</v>
+        <v>364042</v>
       </c>
       <c r="G13" s="23">
-        <v>0.27</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="H13" s="24">
         <f t="shared" si="0"/>
-        <v>-0.77955241417526688</v>
+        <v>-0.44789220920493489</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1847,14 +1861,14 @@
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27">
-        <v>171908</v>
+        <v>351793</v>
       </c>
       <c r="G14" s="28">
         <v>0.22</v>
       </c>
       <c r="H14" s="29">
         <f t="shared" si="0"/>
-        <v>-0.77680046871018682</v>
+        <v>-0.54324387049446654</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1868,7 +1882,9 @@
         <v>17325</v>
       </c>
       <c r="E15" s="22"/>
-      <c r="F15" s="21"/>
+      <c r="F15" s="21">
+        <v>0</v>
+      </c>
       <c r="G15" s="23"/>
       <c r="H15" s="24" t="str">
         <f t="shared" si="0"/>
@@ -1882,7 +1898,9 @@
       <c r="C16" s="26"/>
       <c r="D16" s="27"/>
       <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
+      <c r="F16" s="27">
+        <v>0</v>
+      </c>
       <c r="G16" s="28"/>
       <c r="H16" s="29" t="str">
         <f t="shared" si="0"/>
@@ -1896,7 +1914,9 @@
       <c r="C17" s="30"/>
       <c r="D17" s="31"/>
       <c r="E17" s="22"/>
-      <c r="F17" s="21"/>
+      <c r="F17" s="21">
+        <v>0</v>
+      </c>
       <c r="G17" s="23"/>
       <c r="H17" s="24" t="str">
         <f t="shared" si="0"/>
@@ -1910,7 +1930,9 @@
       <c r="C18" s="26"/>
       <c r="D18" s="27"/>
       <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
+      <c r="F18" s="27">
+        <v>0</v>
+      </c>
       <c r="G18" s="28"/>
       <c r="H18" s="29" t="str">
         <f t="shared" si="0"/>
@@ -1924,7 +1946,9 @@
       <c r="C19" s="30"/>
       <c r="D19" s="31"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="21"/>
+      <c r="F19" s="21">
+        <v>0</v>
+      </c>
       <c r="G19" s="23"/>
       <c r="H19" s="24" t="str">
         <f t="shared" si="0"/>
@@ -1938,7 +1962,9 @@
       <c r="C20" s="26"/>
       <c r="D20" s="27"/>
       <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
+      <c r="F20" s="27">
+        <v>0</v>
+      </c>
       <c r="G20" s="28"/>
       <c r="H20" s="29" t="str">
         <f t="shared" si="0"/>
@@ -1952,7 +1978,9 @@
       <c r="C21" s="30"/>
       <c r="D21" s="31"/>
       <c r="E21" s="22"/>
-      <c r="F21" s="21"/>
+      <c r="F21" s="21">
+        <v>0</v>
+      </c>
       <c r="G21" s="23"/>
       <c r="H21" s="24" t="str">
         <f t="shared" si="0"/>
@@ -1966,7 +1994,9 @@
       <c r="C22" s="26"/>
       <c r="D22" s="27"/>
       <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
+      <c r="F22" s="27">
+        <v>0</v>
+      </c>
       <c r="G22" s="28"/>
       <c r="H22" s="29" t="str">
         <f t="shared" si="0"/>
@@ -1980,7 +2010,9 @@
       <c r="C23" s="30"/>
       <c r="D23" s="31"/>
       <c r="E23" s="22"/>
-      <c r="F23" s="21"/>
+      <c r="F23" s="21">
+        <v>0</v>
+      </c>
       <c r="G23" s="23"/>
       <c r="H23" s="24" t="str">
         <f t="shared" si="0"/>
@@ -1994,7 +2026,9 @@
       <c r="C24" s="26"/>
       <c r="D24" s="27"/>
       <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
+      <c r="F24" s="27">
+        <v>0</v>
+      </c>
       <c r="G24" s="28"/>
       <c r="H24" s="29" t="str">
         <f t="shared" si="0"/>
@@ -2019,27 +2053,27 @@
       </c>
       <c r="F25" s="34">
         <f>SUM(F5:F24)</f>
-        <v>3200387</v>
+        <v>6684729</v>
       </c>
       <c r="G25" s="35">
         <f>IF(F25=0,"-",SUMPRODUCT(F5:F24,G5:G24)/F25)</f>
-        <v>0.32511615001560751</v>
+        <v>0.32573553542709066</v>
       </c>
       <c r="H25" s="35">
         <f>IF(D25=0,"-",(F25-D25)/D25)</f>
-        <v>-0.76101567311789919</v>
+        <v>-0.50082741229286987</v>
       </c>
     </row>
     <row r="28" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="78" t="s">
+      <c r="B28" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="78"/>
-      <c r="D28" s="78"/>
-      <c r="E28" s="78"/>
-      <c r="F28" s="78"/>
-      <c r="G28" s="78"/>
-      <c r="H28" s="78"/>
+      <c r="C28" s="77"/>
+      <c r="D28" s="77"/>
+      <c r="E28" s="77"/>
+      <c r="F28" s="77"/>
+      <c r="G28" s="77"/>
+      <c r="H28" s="77"/>
       <c r="I28" s="36"/>
     </row>
     <row r="29" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2328,7 +2362,7 @@
       </c>
       <c r="H38" s="24">
         <f>H25</f>
-        <v>-0.76101567311789919</v>
+        <v>-0.50082741229286987</v>
       </c>
     </row>
     <row r="39" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2337,7 +2371,7 @@
       </c>
       <c r="H39" s="24">
         <f>G25</f>
-        <v>0.32511615001560751</v>
+        <v>0.32573553542709066</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2376,42 +2410,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="80" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
-      <c r="M1" s="74"/>
-      <c r="N1" s="74"/>
-      <c r="O1" s="74"/>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
+      <c r="O1" s="80"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="75" t="s">
+      <c r="A2" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="75"/>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="75"/>
-      <c r="L2" s="75"/>
-      <c r="M2" s="75"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="75"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="81"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="81"/>
     </row>
     <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
@@ -2495,9 +2529,15 @@
       <c r="E9" s="21">
         <v>5865309</v>
       </c>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
+      <c r="F9" s="21">
+        <v>5850646</v>
+      </c>
+      <c r="G9" s="21">
+        <v>5273394</v>
+      </c>
+      <c r="H9" s="21">
+        <v>6245934</v>
+      </c>
       <c r="I9" s="21"/>
       <c r="J9" s="21"/>
       <c r="K9" s="21"/>
@@ -2506,7 +2546,7 @@
       <c r="N9" s="21"/>
       <c r="O9" s="49">
         <f>SUM(C9:N9)</f>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2520,10 +2560,14 @@
         <v>3378546</v>
       </c>
       <c r="E10" s="21">
-        <v>3965412</v>
-      </c>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
+        <v>3769893</v>
+      </c>
+      <c r="F10" s="21">
+        <v>3695903</v>
+      </c>
+      <c r="G10" s="21">
+        <v>3277815</v>
+      </c>
       <c r="H10" s="21"/>
       <c r="I10" s="21"/>
       <c r="J10" s="21"/>
@@ -2533,7 +2577,7 @@
       <c r="N10" s="21"/>
       <c r="O10" s="49">
         <f>SUM(C10:N10)</f>
-        <v>10698760</v>
+        <v>17476959</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2550,19 +2594,19 @@
       </c>
       <c r="E11" s="50">
         <f t="shared" si="0"/>
-        <v>1899897</v>
+        <v>2095416</v>
       </c>
       <c r="F11" s="50">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2154743</v>
       </c>
       <c r="G11" s="50">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1995579</v>
       </c>
       <c r="H11" s="50">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6245934</v>
       </c>
       <c r="I11" s="50">
         <f t="shared" si="0"/>
@@ -2590,7 +2634,7 @@
       </c>
       <c r="O11" s="39">
         <f t="shared" si="0"/>
-        <v>6052013</v>
+        <v>16643788</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2607,19 +2651,19 @@
       </c>
       <c r="E12" s="51">
         <f t="shared" si="1"/>
-        <v>0.32392104150011536</v>
-      </c>
-      <c r="F12" s="51" t="str">
+        <v>0.3572558581312596</v>
+      </c>
+      <c r="F12" s="51">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="G12" s="51" t="str">
+        <v>0.3682914673012177</v>
+      </c>
+      <c r="G12" s="51">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="H12" s="51" t="str">
+        <v>0.37842402824442856</v>
+      </c>
+      <c r="H12" s="51">
         <f t="shared" si="1"/>
-        <v>-</v>
+        <v>1</v>
       </c>
       <c r="I12" s="51" t="str">
         <f t="shared" si="1"/>
@@ -2647,7 +2691,7 @@
       </c>
       <c r="O12" s="42">
         <f t="shared" si="1"/>
-        <v>0.36129753534359282</v>
+        <v>0.48779084467289063</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2668,43 +2712,43 @@
       </c>
       <c r="F13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>22601419</v>
       </c>
       <c r="G13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>27874813</v>
       </c>
       <c r="H13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="I13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="J13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="K13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="L13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="M13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="N13" s="50">
         <f t="shared" si="2"/>
-        <v>16750773</v>
+        <v>34120747</v>
       </c>
       <c r="O13" s="39">
         <f t="shared" si="2"/>
-        <v>33501546</v>
+        <v>68241494</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2725,43 +2769,43 @@
       </c>
       <c r="F14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.30398450138504157</v>
+        <v>-6.0882867036011132E-2</v>
       </c>
       <c r="G14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.44318760110803324</v>
+        <v>-7.3413418282548437E-2</v>
       </c>
       <c r="H14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.53598966759002775</v>
+        <v>-5.4826952908587259E-2</v>
       </c>
       <c r="I14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.60227685793430941</v>
+        <v>-0.18985167392164617</v>
       </c>
       <c r="J14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.65199225069252076</v>
+        <v>-0.2911202146814405</v>
       </c>
       <c r="K14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.6906597783933518</v>
+        <v>-0.36988463527239152</v>
       </c>
       <c r="L14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.72159380055401656</v>
+        <v>-0.43289617174515233</v>
       </c>
       <c r="M14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.74690345504910605</v>
+        <v>-0.4844510652228658</v>
       </c>
       <c r="N14" s="51">
         <f t="shared" si="3"/>
-        <v>-0.76799483379501388</v>
+        <v>-0.52741347645429359</v>
       </c>
       <c r="O14" s="42">
         <f t="shared" ref="O14" si="4">IF($C$4=0,"-",(O13-$C$4)/$C$4)</f>
-        <v>-0.53598966759002775</v>
+        <v>-5.4826952908587259E-2</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2775,7 +2819,7 @@
       </c>
       <c r="G17" s="24">
         <f>IF(C4=0,"-",(O9-C4)/C4)</f>
-        <v>-0.76799483379501388</v>
+        <v>-0.52741347645429359</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2784,7 +2828,7 @@
       </c>
       <c r="G18" s="24">
         <f>IF(O9=0,"-",O11/O9)</f>
-        <v>0.36129753534359282</v>
+        <v>0.48779084467289063</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2823,22 +2867,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="81" t="s">
+      <c r="A1" s="82" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="83" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="82"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
@@ -2992,26 +3036,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="85" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
+      <c r="B2" s="85"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -3316,7 +3360,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3326,20 +3370,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="86" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="86"/>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
+      <c r="B2" s="87"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
     </row>
     <row r="3" spans="1:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3783,6 +3827,48 @@
         <v>166</v>
       </c>
       <c r="D35" s="70" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>2026</v>
+      </c>
+      <c r="B36" s="74">
+        <v>46154</v>
+      </c>
+      <c r="C36" t="s">
+        <v>167</v>
+      </c>
+      <c r="D36" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>2026</v>
+      </c>
+      <c r="B37" s="74">
+        <v>46155</v>
+      </c>
+      <c r="C37" t="s">
+        <v>168</v>
+      </c>
+      <c r="D37" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>2026</v>
+      </c>
+      <c r="B38" s="74">
+        <v>46185</v>
+      </c>
+      <c r="C38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D38" t="s">
         <v>127</v>
       </c>
     </row>

</xml_diff>